<commit_message>
fix: mejoras del diseño para el reporte del excel
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\senati\FrontEnd-Proyecto_World_Internacional\src\utils\reporte_excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\senati\FrontEnd-Proyecto_World_Internacional\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE81C3C-FCB8-4A52-9BC5-40DEA49A7F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5DE67DF-FA9C-4248-B8CB-95F6130460DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{7629E82F-DF80-4E05-ACE4-DDABCBCA32AB}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -151,11 +150,11 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -478,22 +477,24 @@
     <col min="5" max="5" width="18.5703125" customWidth="1"/>
     <col min="6" max="6" width="17.28515625" customWidth="1"/>
     <col min="7" max="7" width="16.140625" customWidth="1"/>
-    <col min="8" max="10" width="22.85546875" customWidth="1"/>
+    <col min="8" max="8" width="22.85546875" customWidth="1"/>
+    <col min="9" max="9" width="37.42578125" customWidth="1"/>
+    <col min="10" max="10" width="22.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:10" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
     </row>
     <row r="4" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
@@ -510,34 +511,34 @@
       <c r="J4" s="2"/>
     </row>
     <row r="5" spans="1:10" s="1" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="4" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>